<commit_message>
Register the policy issue, return premium and quotation discount approvals in the Authority Matrix; align setting fallbacks with the TISPH values; purge the sample promotions
</commit_message>
<xml_diff>
--- a/docs/package/05_Delivery/Upload_Templates/Endorsement_Type_Upload_Template.xlsx
+++ b/docs/package/05_Delivery/Upload_Templates/Endorsement_Type_Upload_Template.xlsx
@@ -39,22 +39,22 @@
     <t xml:space="preserve">Status</t>
   </si>
   <si>
-    <t xml:space="preserve">CPLT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Change of Plate Number</t>
+    <t xml:space="preserve">CMOB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change of Mobile Number</t>
   </si>
   <si>
     <t xml:space="preserve">No</t>
   </si>
   <si>
-    <t xml:space="preserve">MOTOR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vehicle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">110</t>
+    <t xml:space="preserve">*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">insured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">990</t>
   </si>
   <si>
     <t xml:space="preserve">Column</t>

</xml_diff>